<commit_message>
feat: add style reading and cloning capabilities, implement workbook protection and defined name management
- Introduced style_read.go for reading and cloning cell styles from styles.xml.
- Implemented GetStyle, CopyStyle, and related functions for style management in WorkSheet and Cell.
- Added workbook_protection.go to manage workbook-level protection and defined names.
- Implemented ProtectWorkbook, UnprotectWorkbook, GetWorkbookProtection, SetDefinedName, GetDefinedName, and DeleteDefinedName functions.
- Enhanced XML manipulation for workbook protection and defined names in workbook.xml.
</commit_message>
<xml_diff>
--- a/generated/08_merge.xlsx
+++ b/generated/08_merge.xlsx
@@ -561,7 +561,7 @@
   <rowBreaks count="1" manualBreakCount="1">
     <brk id="2" min="0" max="16383" man="1"/>
   </rowBreaks>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -596,6 +596,6 @@
   <rowBreaks count="1" manualBreakCount="1">
     <brk id="2" min="0" max="16383" man="1"/>
   </rowBreaks>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>